<commit_message>
feat: novos dados de percentil e dados de Brasília
</commit_message>
<xml_diff>
--- a/base_datas/receitas_correntes_detalhamento.xlsx
+++ b/base_datas/receitas_correntes_detalhamento.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D5479"/>
+  <dimension ref="A1:D5480"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -74941,6 +74941,20 @@
         <v>53920007.97</v>
       </c>
     </row>
+    <row r="5480">
+      <c r="A5480">
+        <v>5300108</v>
+      </c>
+      <c r="B5480">
+        <v>24842769006.59</v>
+      </c>
+      <c r="C5480">
+        <v>2751796117.43</v>
+      </c>
+      <c r="D5480">
+        <v>7076164310.14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: adiciona dados de brasília e suas respectivas receitas
</commit_message>
<xml_diff>
--- a/base_datas/receitas_correntes_detalhamento.xlsx
+++ b/base_datas/receitas_correntes_detalhamento.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D5479"/>
+  <dimension ref="A1:D5480"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -74941,6 +74941,20 @@
         <v>53920007.97</v>
       </c>
     </row>
+    <row r="5480">
+      <c r="A5480">
+        <v>5300108</v>
+      </c>
+      <c r="B5480">
+        <v>24842769006.59</v>
+      </c>
+      <c r="C5480">
+        <v>2751796117.43</v>
+      </c>
+      <c r="D5480">
+        <v>7076164310.14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>